<commit_message>
improved doc on compute methods and others
</commit_message>
<xml_diff>
--- a/mario/settings/Terminology.xlsx
+++ b/mario/settings/Terminology.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365.sharepoint.com/sites/DENG-SESAM/Documenti condivisi/c-Research/b-Models/MARIO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzorinaldi/Documents/GitHub/MARIO/mario/settings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="8_{C61CA938-AF74-E241-ABEE-A9877181FB2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{351B3BC4-5470-B242-8ECC-8CA440EB678A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1528DB09-E247-F441-859B-1F63CA009EFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26880" activeTab="1" xr2:uid="{191C6CC1-D0C2-3B4B-A0D5-6A4A3794157A}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17660" xr2:uid="{191C6CC1-D0C2-3B4B-A0D5-6A4A3794157A}"/>
   </bookViews>
   <sheets>
     <sheet name="Matrices" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="164">
   <si>
     <t>Also known as</t>
   </si>
@@ -496,6 +496,42 @@
   </si>
   <si>
     <t>Environmental extensions</t>
+  </si>
+  <si>
+    <t>bu</t>
+  </si>
+  <si>
+    <t>bs</t>
+  </si>
+  <si>
+    <t>Use transaction direct-output coefficients matrix</t>
+  </si>
+  <si>
+    <t>Supply transaction direct-output coefficients matrix</t>
+  </si>
+  <si>
+    <t>gcc</t>
+  </si>
+  <si>
+    <t>gca</t>
+  </si>
+  <si>
+    <t>gac</t>
+  </si>
+  <si>
+    <t>gaa</t>
+  </si>
+  <si>
+    <t>Ghosh inverse matrix, commodity-by-commodity coefficients</t>
+  </si>
+  <si>
+    <t>Ghosh inverse matrix, commodity-by-activity coefficients</t>
+  </si>
+  <si>
+    <t>Ghosh inverse matrix, activity-by-commodity coefficients</t>
+  </si>
+  <si>
+    <t>Ghosh inverse matrix, activity-by-activity coefficients</t>
   </si>
 </sst>
 </file>
@@ -875,7 +911,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15D6DF91-CF4F-D845-84FA-5FC099A8086B}">
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.6640625" customWidth="1"/>
@@ -1905,7 +1941,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>127</v>
       </c>
@@ -1927,7 +1963,7 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B49" t="s">
         <v>14</v>
@@ -1936,10 +1972,10 @@
         <v>8</v>
       </c>
       <c r="D49" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E49" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F49" t="s">
         <v>7</v>
@@ -1950,7 +1986,7 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B50" t="s">
         <v>14</v>
@@ -1959,16 +1995,154 @@
         <v>8</v>
       </c>
       <c r="D50" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E50" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F50" t="s">
         <v>7</v>
       </c>
       <c r="G50" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>152</v>
+      </c>
+      <c r="B51" t="s">
+        <v>14</v>
+      </c>
+      <c r="C51" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" t="s">
+        <v>123</v>
+      </c>
+      <c r="E51" t="s">
+        <v>154</v>
+      </c>
+      <c r="F51" t="s">
+        <v>61</v>
+      </c>
+      <c r="G51" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>153</v>
+      </c>
+      <c r="B52" t="s">
+        <v>14</v>
+      </c>
+      <c r="C52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" t="s">
+        <v>123</v>
+      </c>
+      <c r="E52" t="s">
+        <v>155</v>
+      </c>
+      <c r="F52" t="s">
+        <v>62</v>
+      </c>
+      <c r="G52" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>156</v>
+      </c>
+      <c r="B53" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53" t="s">
+        <v>120</v>
+      </c>
+      <c r="E53" t="s">
+        <v>160</v>
+      </c>
+      <c r="F53" t="s">
+        <v>61</v>
+      </c>
+      <c r="G53" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B54" t="s">
+        <v>14</v>
+      </c>
+      <c r="C54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D54" t="s">
+        <v>120</v>
+      </c>
+      <c r="E54" t="s">
+        <v>161</v>
+      </c>
+      <c r="F54" t="s">
+        <v>61</v>
+      </c>
+      <c r="G54" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>158</v>
+      </c>
+      <c r="B55" t="s">
+        <v>14</v>
+      </c>
+      <c r="C55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D55" t="s">
+        <v>120</v>
+      </c>
+      <c r="E55" t="s">
+        <v>162</v>
+      </c>
+      <c r="F55" t="s">
+        <v>62</v>
+      </c>
+      <c r="G55" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>159</v>
+      </c>
+      <c r="B56" t="s">
+        <v>14</v>
+      </c>
+      <c r="C56" t="s">
+        <v>9</v>
+      </c>
+      <c r="D56" t="s">
+        <v>120</v>
+      </c>
+      <c r="E56" t="s">
+        <v>163</v>
+      </c>
+      <c r="F56" t="s">
+        <v>62</v>
+      </c>
+      <c r="G56" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -2109,6 +2283,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100241E96938535DD4B921FCDFB54345D30" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c3c32a72d805f5b6b1b477f46f0cbd5b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e" xmlns:ns3="e67e9a88-35e1-4b39-8da9-a609eb308282" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8adfbf54647c461499df9b7ce19975bb" ns2:_="" ns3:_="">
     <xsd:import namespace="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
@@ -2369,15 +2552,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2390,13 +2564,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C513B84B-7C74-48D1-86D3-A26BEDAA5B47}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB3399AB-9254-4941-8CB3-3E5BD94FC575}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB3399AB-9254-4941-8CB3-3E5BD94FC575}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C513B84B-7C74-48D1-86D3-A26BEDAA5B47}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
+    <ds:schemaRef ds:uri="e67e9a88-35e1-4b39-8da9-a609eb308282"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8F939E8-3FDD-4B79-B7F8-18DD0CA0CBEC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8F939E8-3FDD-4B79-B7F8-18DD0CA0CBEC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
+    <ds:schemaRef ds:uri="e67e9a88-35e1-4b39-8da9-a609eb308282"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fixed isard_to_chenery and terminology updated
</commit_message>
<xml_diff>
--- a/mario/settings/Terminology.xlsx
+++ b/mario/settings/Terminology.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzorinaldi/Documents/GitHub/MARIO/mario/settings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1528DB09-E247-F441-859B-1F63CA009EFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F51F109-E964-2B45-B6E1-4478D26C55D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17660" xr2:uid="{191C6CC1-D0C2-3B4B-A0D5-6A4A3794157A}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="180">
   <si>
     <t>Also known as</t>
   </si>
@@ -532,6 +532,54 @@
   </si>
   <si>
     <t>Ghosh inverse matrix, activity-by-activity coefficients</t>
+  </si>
+  <si>
+    <t>mc_ex</t>
+  </si>
+  <si>
+    <t>Total (direct+indirect) value added coefficients by commodity matrix, exploded by origin region and activity</t>
+  </si>
+  <si>
+    <t>Factor of production, Region, Activity</t>
+  </si>
+  <si>
+    <t>ma_ex</t>
+  </si>
+  <si>
+    <t>Total (direct+indirect) value added coefficients by activity matrix, exploded by origin region and activity</t>
+  </si>
+  <si>
+    <t>fc_ex</t>
+  </si>
+  <si>
+    <t>Total (direct+indirect) environmental coefficients by commodity matrix, exploded by origin region and activity</t>
+  </si>
+  <si>
+    <t>Satellite account, Region, Activity</t>
+  </si>
+  <si>
+    <t>fa_ex</t>
+  </si>
+  <si>
+    <t>Total (direct+indirect) environmental coefficients by activity matrix, exploded by origin region and activity</t>
+  </si>
+  <si>
+    <t>m_ex</t>
+  </si>
+  <si>
+    <t>Total (direct+indirect) value added coefficients matrix, exploded by origin region and sector</t>
+  </si>
+  <si>
+    <t>Factor of production, Region, Sector</t>
+  </si>
+  <si>
+    <t>f_ex</t>
+  </si>
+  <si>
+    <t>Total (direct+indirect) environmental coefficients matrix, exploded by origin region and sector</t>
+  </si>
+  <si>
+    <t>Satellite account, Region, Sector</t>
   </si>
 </sst>
 </file>
@@ -911,7 +959,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15D6DF91-CF4F-D845-84FA-5FC099A8086B}">
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.6640625" customWidth="1"/>
@@ -1241,22 +1289,19 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>174</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C15" t="s">
         <v>8</v>
       </c>
-      <c r="D15" t="s">
-        <v>54</v>
-      </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>175</v>
       </c>
       <c r="F15" t="s">
-        <v>47</v>
+        <v>176</v>
       </c>
       <c r="G15" t="s">
         <v>7</v>
@@ -1264,19 +1309,19 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C16" t="s">
         <v>8</v>
       </c>
       <c r="D16" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="E16" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F16" t="s">
         <v>47</v>
@@ -1287,7 +1332,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
@@ -1295,65 +1340,62 @@
       <c r="C17" t="s">
         <v>8</v>
       </c>
+      <c r="D17" t="s">
+        <v>44</v>
+      </c>
       <c r="E17" t="s">
-        <v>128</v>
+        <v>53</v>
       </c>
       <c r="F17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17" t="s">
         <v>7</v>
-      </c>
-      <c r="G17" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>55</v>
+        <v>177</v>
       </c>
       <c r="B18" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E18" t="s">
-        <v>60</v>
+        <v>178</v>
       </c>
       <c r="F18" t="s">
-        <v>61</v>
+        <v>179</v>
       </c>
       <c r="G18" t="s">
-        <v>62</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>125</v>
       </c>
       <c r="B19" t="s">
         <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E19" t="s">
-        <v>63</v>
+        <v>128</v>
       </c>
       <c r="F19" t="s">
-        <v>61</v>
+        <v>7</v>
       </c>
       <c r="G19" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B20" t="s">
         <v>12</v>
@@ -1362,21 +1404,21 @@
         <v>9</v>
       </c>
       <c r="D20" t="s">
-        <v>59</v>
+        <v>5</v>
       </c>
       <c r="E20" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F20" t="s">
+        <v>61</v>
+      </c>
+      <c r="G20" t="s">
         <v>62</v>
-      </c>
-      <c r="G20" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
@@ -1388,38 +1430,41 @@
         <v>15</v>
       </c>
       <c r="E21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F21" t="s">
+        <v>61</v>
+      </c>
+      <c r="G21" t="s">
         <v>62</v>
-      </c>
-      <c r="G21" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="B22" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C22" t="s">
         <v>9</v>
       </c>
+      <c r="D22" t="s">
+        <v>59</v>
+      </c>
       <c r="E22" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F22" t="s">
+        <v>62</v>
+      </c>
+      <c r="G22" t="s">
         <v>61</v>
-      </c>
-      <c r="G22" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>111</v>
+        <v>58</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -1428,13 +1473,13 @@
         <v>9</v>
       </c>
       <c r="D23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E23" t="s">
-        <v>115</v>
+        <v>66</v>
       </c>
       <c r="F23" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G23" t="s">
         <v>61</v>
@@ -1442,7 +1487,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>112</v>
+        <v>65</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
@@ -1450,11 +1495,8 @@
       <c r="C24" t="s">
         <v>9</v>
       </c>
-      <c r="D24" t="s">
-        <v>16</v>
-      </c>
       <c r="E24" t="s">
-        <v>116</v>
+        <v>67</v>
       </c>
       <c r="F24" t="s">
         <v>61</v>
@@ -1465,7 +1507,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
@@ -1477,10 +1519,10 @@
         <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G25" t="s">
         <v>61</v>
@@ -1488,7 +1530,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
@@ -1500,10 +1542,10 @@
         <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F26" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G26" t="s">
         <v>62</v>
@@ -1511,53 +1553,53 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="B27" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C27" t="s">
         <v>9</v>
       </c>
       <c r="D27" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E27" t="s">
-        <v>70</v>
+        <v>117</v>
       </c>
       <c r="F27" t="s">
+        <v>62</v>
+      </c>
+      <c r="G27" t="s">
         <v>61</v>
-      </c>
-      <c r="G27" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>69</v>
+        <v>114</v>
       </c>
       <c r="B28" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C28" t="s">
         <v>9</v>
       </c>
       <c r="D28" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>71</v>
+        <v>118</v>
       </c>
       <c r="F28" t="s">
         <v>62</v>
       </c>
       <c r="G28" t="s">
-        <v>23</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B29" t="s">
         <v>12</v>
@@ -1566,21 +1608,21 @@
         <v>9</v>
       </c>
       <c r="D29" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="E29" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="F29" t="s">
         <v>61</v>
       </c>
       <c r="G29" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B30" t="s">
         <v>12</v>
@@ -1589,21 +1631,21 @@
         <v>9</v>
       </c>
       <c r="D30" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E30" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F30" t="s">
         <v>62</v>
       </c>
       <c r="G30" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B31" t="s">
         <v>12</v>
@@ -1611,19 +1653,22 @@
       <c r="C31" t="s">
         <v>9</v>
       </c>
+      <c r="D31" t="s">
+        <v>74</v>
+      </c>
       <c r="E31" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="F31" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="G31" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B32" t="s">
         <v>12</v>
@@ -1631,28 +1676,31 @@
       <c r="C32" t="s">
         <v>9</v>
       </c>
+      <c r="D32" t="s">
+        <v>24</v>
+      </c>
       <c r="E32" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F32" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="G32" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B33" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C33" t="s">
         <v>9</v>
       </c>
       <c r="E33" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F33" t="s">
         <v>46</v>
@@ -1663,16 +1711,16 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="B34" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C34" t="s">
         <v>9</v>
       </c>
       <c r="E34" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="F34" t="s">
         <v>46</v>
@@ -1683,19 +1731,19 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B35" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C35" t="s">
         <v>9</v>
       </c>
       <c r="E35" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="F35" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G35" t="s">
         <v>61</v>
@@ -1703,19 +1751,19 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B36" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C36" t="s">
         <v>9</v>
       </c>
       <c r="E36" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="F36" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G36" t="s">
         <v>62</v>
@@ -1723,16 +1771,16 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B37" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C37" t="s">
         <v>9</v>
       </c>
       <c r="E37" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F37" t="s">
         <v>47</v>
@@ -1743,16 +1791,16 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B38" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C38" t="s">
         <v>9</v>
       </c>
       <c r="E38" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F38" t="s">
         <v>47</v>
@@ -1763,19 +1811,19 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="B39" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C39" t="s">
         <v>9</v>
       </c>
       <c r="E39" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="F39" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G39" t="s">
         <v>61</v>
@@ -1783,19 +1831,19 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B40" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C40" t="s">
         <v>9</v>
       </c>
       <c r="E40" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="F40" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G40" t="s">
         <v>62</v>
@@ -1803,16 +1851,16 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B41" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C41" t="s">
         <v>9</v>
       </c>
       <c r="E41" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F41" t="s">
         <v>46</v>
@@ -1823,16 +1871,16 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B42" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C42" t="s">
         <v>9</v>
       </c>
       <c r="E42" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F42" t="s">
         <v>46</v>
@@ -1843,19 +1891,19 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B43" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C43" t="s">
         <v>9</v>
       </c>
       <c r="E43" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F43" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G43" t="s">
         <v>61</v>
@@ -1863,19 +1911,19 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B44" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C44" t="s">
         <v>9</v>
       </c>
       <c r="E44" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G44" t="s">
         <v>62</v>
@@ -1883,19 +1931,19 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>101</v>
+        <v>164</v>
       </c>
       <c r="B45" t="s">
         <v>14</v>
       </c>
       <c r="C45" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E45" t="s">
-        <v>109</v>
+        <v>165</v>
       </c>
       <c r="F45" t="s">
-        <v>47</v>
+        <v>166</v>
       </c>
       <c r="G45" t="s">
         <v>61</v>
@@ -1903,19 +1951,19 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>102</v>
+        <v>167</v>
       </c>
       <c r="B46" t="s">
         <v>14</v>
       </c>
       <c r="C46" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E46" t="s">
-        <v>110</v>
+        <v>168</v>
       </c>
       <c r="F46" t="s">
-        <v>47</v>
+        <v>166</v>
       </c>
       <c r="G46" t="s">
         <v>62</v>
@@ -1923,139 +1971,127 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="B47" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C47" t="s">
         <v>9</v>
       </c>
       <c r="E47" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
       <c r="F47" t="s">
+        <v>47</v>
+      </c>
+      <c r="G47" t="s">
         <v>61</v>
       </c>
-      <c r="G47" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="B48" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C48" t="s">
         <v>9</v>
       </c>
       <c r="E48" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="F48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G48" t="s">
         <v>62</v>
-      </c>
-      <c r="G48" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="B49" t="s">
         <v>14</v>
       </c>
       <c r="C49" t="s">
-        <v>8</v>
-      </c>
-      <c r="D49" t="s">
-        <v>123</v>
+        <v>9</v>
       </c>
       <c r="E49" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="F49" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="G49" t="s">
-        <v>7</v>
+        <v>61</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="B50" t="s">
         <v>14</v>
       </c>
       <c r="C50" t="s">
-        <v>8</v>
-      </c>
-      <c r="D50" t="s">
-        <v>120</v>
+        <v>9</v>
       </c>
       <c r="E50" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="F50" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="G50" t="s">
-        <v>7</v>
+        <v>62</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="B51" t="s">
         <v>14</v>
       </c>
       <c r="C51" t="s">
-        <v>9</v>
-      </c>
-      <c r="D51" t="s">
-        <v>123</v>
+        <v>8</v>
       </c>
       <c r="E51" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="F51" t="s">
+        <v>171</v>
+      </c>
+      <c r="G51" t="s">
         <v>61</v>
-      </c>
-      <c r="G51" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="B52" t="s">
         <v>14</v>
       </c>
       <c r="C52" t="s">
-        <v>9</v>
-      </c>
-      <c r="D52" t="s">
-        <v>123</v>
+        <v>8</v>
       </c>
       <c r="E52" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="F52" t="s">
+        <v>171</v>
+      </c>
+      <c r="G52" t="s">
         <v>62</v>
-      </c>
-      <c r="G52" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>156</v>
+        <v>126</v>
       </c>
       <c r="B53" t="s">
         <v>14</v>
@@ -2063,22 +2099,19 @@
       <c r="C53" t="s">
         <v>9</v>
       </c>
-      <c r="D53" t="s">
-        <v>120</v>
-      </c>
       <c r="E53" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="F53" t="s">
         <v>61</v>
       </c>
       <c r="G53" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>157</v>
+        <v>127</v>
       </c>
       <c r="B54" t="s">
         <v>14</v>
@@ -2086,62 +2119,197 @@
       <c r="C54" t="s">
         <v>9</v>
       </c>
-      <c r="D54" t="s">
-        <v>120</v>
-      </c>
       <c r="E54" t="s">
-        <v>161</v>
+        <v>130</v>
       </c>
       <c r="F54" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G54" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>158</v>
+        <v>124</v>
       </c>
       <c r="B55" t="s">
         <v>14</v>
       </c>
       <c r="C55" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D55" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E55" t="s">
-        <v>162</v>
+        <v>122</v>
       </c>
       <c r="F55" t="s">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="G55" t="s">
-        <v>61</v>
+        <v>7</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>159</v>
+        <v>119</v>
       </c>
       <c r="B56" t="s">
         <v>14</v>
       </c>
       <c r="C56" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D56" t="s">
         <v>120</v>
       </c>
       <c r="E56" t="s">
+        <v>121</v>
+      </c>
+      <c r="F56" t="s">
+        <v>7</v>
+      </c>
+      <c r="G56" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>152</v>
+      </c>
+      <c r="B57" t="s">
+        <v>14</v>
+      </c>
+      <c r="C57" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" t="s">
+        <v>123</v>
+      </c>
+      <c r="E57" t="s">
+        <v>154</v>
+      </c>
+      <c r="F57" t="s">
+        <v>61</v>
+      </c>
+      <c r="G57" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>153</v>
+      </c>
+      <c r="B58" t="s">
+        <v>14</v>
+      </c>
+      <c r="C58" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58" t="s">
+        <v>123</v>
+      </c>
+      <c r="E58" t="s">
+        <v>155</v>
+      </c>
+      <c r="F58" t="s">
+        <v>62</v>
+      </c>
+      <c r="G58" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>156</v>
+      </c>
+      <c r="B59" t="s">
+        <v>14</v>
+      </c>
+      <c r="C59" t="s">
+        <v>9</v>
+      </c>
+      <c r="D59" t="s">
+        <v>120</v>
+      </c>
+      <c r="E59" t="s">
+        <v>160</v>
+      </c>
+      <c r="F59" t="s">
+        <v>61</v>
+      </c>
+      <c r="G59" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>157</v>
+      </c>
+      <c r="B60" t="s">
+        <v>14</v>
+      </c>
+      <c r="C60" t="s">
+        <v>9</v>
+      </c>
+      <c r="D60" t="s">
+        <v>120</v>
+      </c>
+      <c r="E60" t="s">
+        <v>161</v>
+      </c>
+      <c r="F60" t="s">
+        <v>61</v>
+      </c>
+      <c r="G60" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>158</v>
+      </c>
+      <c r="B61" t="s">
+        <v>14</v>
+      </c>
+      <c r="C61" t="s">
+        <v>9</v>
+      </c>
+      <c r="D61" t="s">
+        <v>120</v>
+      </c>
+      <c r="E61" t="s">
+        <v>162</v>
+      </c>
+      <c r="F61" t="s">
+        <v>62</v>
+      </c>
+      <c r="G61" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>159</v>
+      </c>
+      <c r="B62" t="s">
+        <v>14</v>
+      </c>
+      <c r="C62" t="s">
+        <v>9</v>
+      </c>
+      <c r="D62" t="s">
+        <v>120</v>
+      </c>
+      <c r="E62" t="s">
         <v>163</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F62" t="s">
         <v>62</v>
       </c>
-      <c r="G56" t="s">
+      <c r="G62" t="s">
         <v>62</v>
       </c>
     </row>
@@ -2283,12 +2451,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="e67e9a88-35e1-4b39-8da9-a609eb308282" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2553,20 +2723,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="e67e9a88-35e1-4b39-8da9-a609eb308282" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB3399AB-9254-4941-8CB3-3E5BD94FC575}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8F939E8-3FDD-4B79-B7F8-18DD0CA0CBEC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
+    <ds:schemaRef ds:uri="e67e9a88-35e1-4b39-8da9-a609eb308282"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2591,12 +2762,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8F939E8-3FDD-4B79-B7F8-18DD0CA0CBEC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB3399AB-9254-4941-8CB3-3E5BD94FC575}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
-    <ds:schemaRef ds:uri="e67e9a88-35e1-4b39-8da9-a609eb308282"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>